<commit_message>
Add Table3 as a sheet to statistical_tests_full150.xlsx
</commit_message>
<xml_diff>
--- a/eval/results/statistical_tests_full150.xlsx
+++ b/eval/results/statistical_tests_full150.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Paired Tests" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Fisher Exact Test" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Table3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16673,4 +16674,650 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>QID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>base_prec</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>FT_prec</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>QSP_prec</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>base_rec</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>FT_rec</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>QSP_rec</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Does the paper report in vitro drug susceptibility data?</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>50.9</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>89.3***</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>92.6</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>97.0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>94.3</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>83.3</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>69.6</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>90.2***</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>92.4***</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>From what years were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>95.7</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>94.1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>85.3</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>78.8</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>94.1**</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>95.3**</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Which HIV genes were reported to have been sequenced?</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>98.8</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>95.0</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>96.8</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>63.5</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>76.2*†</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>73.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>11</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>88.9</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>92.7</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>87.3</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>60.9</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>82.6**</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>14</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>96.6</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>89.3</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>91.0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>76.7</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>91.8*†</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>83.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>15</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>64.9</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>86.4**</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>70.7</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>74.6</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>85.1</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>61.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>55.6</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>80.7**</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>52.6</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>80.7**</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>29.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Llama3.1-70B</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>From which countries were the sequenced samples obtained?</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>87.7</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>96.1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>97.6*†</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>77.2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Llama3.1-70B</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>11</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>What type of samples were sequenced?</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>86.2</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>96.9*†</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>89.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>68.5</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Llama3.1-70B</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>14</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>77.0</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>98.1***</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>88.6</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>78.1</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>71.2</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>84.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Llama3.1-70B</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>47.9</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>77.1***</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>78.3***</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>86.6</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>55.2</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>70.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Llama3.1-70B</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>16</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>38.9</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>70.6**</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>68.3**</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>73.7</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>49.1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
provide BH summary, update Table3 and restrict p-values in bar chart
</commit_message>
<xml_diff>
--- a/eval/results/statistical_tests_full150.xlsx
+++ b/eval/results/statistical_tests_full150.xlsx
@@ -24746,7 +24746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24803,41 +24803,41 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from patient samples?</t>
+          <t>Does the paper report in vitro drug susceptibility data?</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>91.7</t>
+          <t>50.9</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>94.1</t>
+          <t>89.3***</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>94.2</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>86.3</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>94.1</t>
+          <t>92.6</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>95.1</t>
+          <t>100.0</t>
         </is>
       </c>
     </row>
@@ -24848,41 +24848,41 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Does the paper report in vitro drug susceptibility data?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>50.9</t>
+          <t>96.9</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>89.3***</t>
+          <t>94.3</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>85.7</t>
+          <t>83.3</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>68.5</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>92.6</t>
+          <t>90.2***</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>88.9</t>
+          <t>92.4***</t>
         </is>
       </c>
     </row>
@@ -24893,41 +24893,41 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>96.9</t>
+          <t>95.7</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>94.3</t>
+          <t>94.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>88.3</t>
+          <t>85.3</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>68.5</t>
+          <t>78.8</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>90.2***</t>
+          <t>92.9*†</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>90.2***</t>
+          <t>95.3**</t>
         </is>
       </c>
     </row>
@@ -24938,41 +24938,41 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>95.7</t>
+          <t>88.7</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>94.0</t>
+          <t>92.6</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>89.7</t>
+          <t>87.3</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>59.8</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>92.9*†</t>
+          <t>81.5**</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>91.8**</t>
+          <t>75.0*†</t>
         </is>
       </c>
     </row>
@@ -24983,41 +24983,41 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>98.7</t>
+          <t>63.5</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>94.8</t>
+          <t>85.9**</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>96.0</t>
+          <t>70.7</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>60.3</t>
+          <t>70.1</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>73.0*†</t>
+          <t>82.1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>61.2</t>
         </is>
       </c>
     </row>
@@ -25028,176 +25028,176 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>88.7</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>92.6</t>
+          <t>78.0**</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>92.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>59.8</t>
+          <t>43.9</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>81.5**</t>
+          <t>68.4*†</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>87.0*†</t>
+          <t>29.8</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GPT-4o</t>
+          <t>Llama3.1-70B</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Does the paper report HIV sequences from patient samples?</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>96.6</t>
+          <t>91.5</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>89.3</t>
+          <t>92.2</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>79.5</t>
+          <t>89.6</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>76.7</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>91.8*†</t>
+          <t>81.4</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>90.4</t>
+          <t>93.1***</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GPT-4o</t>
+          <t>Llama3.1-70B</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>63.5</t>
+          <t>77.0</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>85.9**</t>
+          <t>98.1***</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>76.8</t>
+          <t>88.6</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>70.1</t>
+          <t>78.1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>82.1</t>
+          <t>71.2</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>64.2</t>
+          <t>84.9</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GPT-4o</t>
+          <t>Llama3.1-70B</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>47.5</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>78.0**</t>
+          <t>77.1***</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>64.3</t>
+          <t>78.3***</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>43.9</t>
+          <t>85.1</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>68.4*†</t>
+          <t>55.2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>47.4</t>
+          <t>70.1</t>
         </is>
       </c>
     </row>
@@ -25208,806 +25208,311 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from patient samples?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>91.5</t>
+          <t>36.5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>92.2</t>
+          <t>69.7**</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>89.6</t>
+          <t>68.3***</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>81.4</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>93.1***</t>
+          <t>49.1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Llama3.1-70B</t>
+          <t>Llama3.1-8B</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>Does the paper report HIV sequences from patient samples?</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>87.5</t>
+          <t>93.1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>96.1</t>
+          <t>91.4</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>97.5*†</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>76.1</t>
+          <t>79.4</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>85.9</t>
+          <t>100.0***</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Llama3.1-70B</t>
+          <t>Llama3.1-8B</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>88.6</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>94.4</t>
+          <t>93.3</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>94.0</t>
+          <t>84.9</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>82.4</t>
+          <t>47.8</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>60.9</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>92.9</t>
+          <t>79.3***</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Llama3.1-70B</t>
+          <t>Llama3.1-8B</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>What method was used for sequencing?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>98.0</t>
+          <t>92.4</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>96.8</t>
+          <t>96.4</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>95.6</t>
+          <t>79.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>61.7</t>
+          <t>71.8</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>75.3</t>
+          <t>62.4</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>80.2*†</t>
+          <t>97.6***</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Llama3.1-70B</t>
+          <t>Llama3.1-8B</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>86.2</t>
+          <t>97.1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>96.9*†</t>
+          <t>98.3</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>88.9</t>
+          <t>94.3</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>53.2</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>68.5</t>
+          <t>46.8</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>78.3</t>
+          <t>78.6***</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Llama3.1-70B</t>
+          <t>Llama3.1-8B</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>85.7</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>98.1***</t>
+          <t>92.3</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>88.6</t>
+          <t>69.1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>78.1</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>71.2</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>84.9</t>
+          <t>91.8***</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Llama3.1-70B</t>
+          <t>Llama3.1-8B</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>47.5</t>
+          <t>76.1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>77.1***</t>
+          <t>88.9</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>78.3***</t>
+          <t>65.1</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>85.1</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>55.2</t>
+          <t>65.8</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>70.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Llama3.1-70B</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>16</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>36.5</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>69.7**</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>68.3***</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>66.7</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>40.4</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>49.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Llama3.1-8B</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from patient samples?</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>93.1</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>91.4</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>73.8</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>79.4</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>72.5</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>88.2***</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Llama3.1-8B</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Does the paper report in vitro drug susceptibility data?</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>59.1</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>87.5*†</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>35.1</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>96.3</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>77.8</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>74.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Llama3.1-8B</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>5</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>94.1</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>95.5</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>81.4</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>63.4</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>62.4</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>56.4*</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Llama3.1-8B</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>6</v>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>93.3</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>92.7</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>47.8</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>60.9</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>55.4***</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Llama3.1-8B</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>7</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>From what years were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>92.4</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>96.4</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>89.7</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>71.8</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>62.4</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>61.2***</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Llama3.1-8B</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>9</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>97.1</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>98.3</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>95.2</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>53.2</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>46.8</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>46.8***</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Llama3.1-8B</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>12</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>85.7</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>92.3</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>70.4</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>59.0</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>59.0</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>62.3***</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Llama3.1-8B</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>14</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>76.1</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>88.9</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>69.1</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>74.0</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>65.8</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>64.4***</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Llama3.1-8B</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>15</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>55.4</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>73.1*†</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>63.3</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>68.7</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>56.7</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>46.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Llama3.1-8B</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>16</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>37.9</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>57.1</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>43.9</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>28.1</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>28.1</t>
+          <t>97.3***</t>
         </is>
       </c>
     </row>

</xml_diff>